<commit_message>
🔥 Dados MIBGAS atualizados automaticamente
</commit_message>
<xml_diff>
--- a/Tarifarios_🔥_Gas_Natural_Tiago_Felicia.xlsx
+++ b/Tarifarios_🔥_Gas_Natural_Tiago_Felicia.xlsx
@@ -13035,7 +13035,7 @@
         <v>46084</v>
       </c>
       <c r="B428" t="n">
-        <v>30.12</v>
+        <v>42.92</v>
       </c>
     </row>
     <row r="429">
@@ -21343,7 +21343,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>